<commit_message>
France daily ratings for 2026-03-30
</commit_message>
<xml_diff>
--- a/output/daily_ratings/france_ratings_2026-03-30.xlsx
+++ b/output/daily_ratings/france_ratings_2026-03-30.xlsx
@@ -588,10 +588,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S2" t="n">
-        <v>106.5608102699606</v>
+        <v>88.28054384115993</v>
       </c>
       <c r="T2" t="n">
-        <v>106.5608102699606</v>
+        <v>88.28054384115993</v>
       </c>
     </row>
     <row r="3">
@@ -662,10 +662,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S3" t="n">
-        <v>95.95742081611307</v>
+        <v>78.55044868032594</v>
       </c>
       <c r="T3" t="n">
-        <v>95.95742081611307</v>
+        <v>78.55044868032594</v>
       </c>
     </row>
     <row r="4">
@@ -736,10 +736,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S4" t="n">
-        <v>98.30825086707641</v>
+        <v>80.70766455949196</v>
       </c>
       <c r="T4" t="n">
-        <v>98.30825086707641</v>
+        <v>80.70766455949196</v>
       </c>
     </row>
     <row r="5">
@@ -810,10 +810,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S5" t="n">
-        <v>100.4708495766566</v>
+        <v>82.69215181524177</v>
       </c>
       <c r="T5" t="n">
-        <v>100.4708495766566</v>
+        <v>82.69215181524177</v>
       </c>
     </row>
     <row r="6">
@@ -884,10 +884,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S6" t="n">
-        <v>99.21734844498627</v>
+        <v>81.54188893482478</v>
       </c>
       <c r="T6" t="n">
-        <v>99.21734844498627</v>
+        <v>81.54188893482478</v>
       </c>
     </row>
     <row r="7">
@@ -958,10 +958,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S7" t="n">
-        <v>99.50503864522855</v>
+        <v>81.80588499357381</v>
       </c>
       <c r="T7" t="n">
-        <v>99.50503864522855</v>
+        <v>81.80588499357381</v>
       </c>
     </row>
     <row r="8">
@@ -1032,10 +1032,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S8" t="n">
-        <v>95.82262135640613</v>
+        <v>78.42675129315683</v>
       </c>
       <c r="T8" t="n">
-        <v>95.82262135640613</v>
+        <v>78.42675129315683</v>
       </c>
     </row>
     <row r="9">
@@ -1106,10 +1106,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S9" t="n">
-        <v>95.22258673140904</v>
+        <v>77.87613547107189</v>
       </c>
       <c r="T9" t="n">
-        <v>95.22258673140904</v>
+        <v>77.87613547107189</v>
       </c>
     </row>
     <row r="10">
@@ -1180,10 +1180,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S10" t="n">
-        <v>90.09843696953313</v>
+        <v>73.17401026682168</v>
       </c>
       <c r="T10" t="n">
-        <v>90.09843696953313</v>
+        <v>73.17401026682168</v>
       </c>
     </row>
     <row r="11">
@@ -1254,10 +1254,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S11" t="n">
-        <v>95.2439594840795</v>
+        <v>77.89574796557072</v>
       </c>
       <c r="T11" t="n">
-        <v>95.2439594840795</v>
+        <v>77.89574796557072</v>
       </c>
     </row>
     <row r="12">
@@ -1328,10 +1328,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S12" t="n">
-        <v>87.43526249381497</v>
+        <v>70.73017462431976</v>
       </c>
       <c r="T12" t="n">
-        <v>87.43526249381497</v>
+        <v>70.73017462431976</v>
       </c>
     </row>
     <row r="13">
@@ -1402,10 +1402,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S13" t="n">
-        <v>89.26414402596993</v>
+        <v>72.40842962223481</v>
       </c>
       <c r="T13" t="n">
-        <v>89.26414402596993</v>
+        <v>72.40842962223481</v>
       </c>
     </row>
     <row r="14">
@@ -1476,10 +1476,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S14" t="n">
-        <v>92.41392641964872</v>
+        <v>75.29879619415142</v>
       </c>
       <c r="T14" t="n">
-        <v>92.41392641964872</v>
+        <v>75.29879619415142</v>
       </c>
     </row>
     <row r="15">
@@ -1550,10 +1550,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S15" t="n">
-        <v>81.42010643485763</v>
+        <v>65.21042632914755</v>
       </c>
       <c r="T15" t="n">
-        <v>81.42010643485763</v>
+        <v>65.21042632914755</v>
       </c>
     </row>
     <row r="16">
@@ -1624,10 +1624,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S16" t="n">
-        <v>78.46924175889718</v>
+        <v>62.50259462789658</v>
       </c>
       <c r="T16" t="n">
-        <v>78.46924175889718</v>
+        <v>62.50259462789658</v>
       </c>
     </row>
     <row r="17">
@@ -1700,10 +1700,10 @@
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>73.84307862124567</v>
+        <v>58.25744191000239</v>
       </c>
       <c r="T17" t="n">
-        <v>73.84307862124567</v>
+        <v>58.25744191000239</v>
       </c>
     </row>
     <row r="18">
@@ -1774,10 +1774,10 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>76.28941121098063</v>
+        <v>60.5022947466143</v>
       </c>
       <c r="T18" t="n">
-        <v>76.28941121098063</v>
+        <v>60.5022947466143</v>
       </c>
     </row>
     <row r="19">
@@ -1848,10 +1848,10 @@
         <v>0</v>
       </c>
       <c r="S19" t="n">
-        <v>69.61076260044165</v>
+        <v>54.37369909244489</v>
       </c>
       <c r="T19" t="n">
-        <v>69.61076260044165</v>
+        <v>54.37369909244489</v>
       </c>
     </row>
     <row r="20">
@@ -1922,10 +1922,10 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>69.40922374230811</v>
+        <v>54.18875895827549</v>
       </c>
       <c r="T20" t="n">
-        <v>69.40922374230811</v>
+        <v>54.18875895827549</v>
       </c>
     </row>
     <row r="21">
@@ -1996,10 +1996,10 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>65.3784465796376</v>
+        <v>50.48995627488739</v>
       </c>
       <c r="T21" t="n">
-        <v>65.3784465796376</v>
+        <v>50.48995627488739</v>
       </c>
     </row>
     <row r="22">
@@ -2070,10 +2070,10 @@
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>65.17690772150408</v>
+        <v>50.30501614071798</v>
       </c>
       <c r="T22" t="n">
-        <v>65.17690772150408</v>
+        <v>50.30501614071798</v>
       </c>
     </row>
     <row r="23">
@@ -2144,10 +2144,10 @@
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>67.62324031123904</v>
+        <v>52.54986897732989</v>
       </c>
       <c r="T23" t="n">
-        <v>67.62324031123904</v>
+        <v>52.54986897732989</v>
       </c>
     </row>
     <row r="24">
@@ -2218,10 +2218,10 @@
         <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>56.19797867501247</v>
+        <v>42.06559096021233</v>
       </c>
       <c r="T24" t="n">
-        <v>56.19797867501247</v>
+        <v>42.06559096021233</v>
       </c>
     </row>
     <row r="25">
@@ -2292,10 +2292,10 @@
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>53.6787429483434</v>
+        <v>39.75383928309477</v>
       </c>
       <c r="T25" t="n">
-        <v>53.6787429483434</v>
+        <v>39.75383928309477</v>
       </c>
     </row>
     <row r="26">
@@ -2366,10 +2366,10 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>53.08457623349256</v>
+        <v>39.2086080905537</v>
       </c>
       <c r="T26" t="n">
-        <v>53.08457623349256</v>
+        <v>39.2086080905537</v>
       </c>
     </row>
     <row r="27">
@@ -2440,10 +2440,10 @@
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>51.57303479749112</v>
+        <v>37.82155708428316</v>
       </c>
       <c r="T27" t="n">
-        <v>51.57303479749112</v>
+        <v>37.82155708428316</v>
       </c>
     </row>
     <row r="28">
@@ -2516,10 +2516,10 @@
         <v>13</v>
       </c>
       <c r="S28" t="n">
-        <v>59.10228155431076</v>
+        <v>44.73069569058723</v>
       </c>
       <c r="T28" t="n">
-        <v>59.10228155431076</v>
+        <v>44.73069569058723</v>
       </c>
     </row>
     <row r="29">
@@ -2590,10 +2590,10 @@
         <v>13</v>
       </c>
       <c r="S29" t="n">
-        <v>57.44092912044468</v>
+        <v>43.20617210805162</v>
       </c>
       <c r="T29" t="n">
-        <v>57.44092912044468</v>
+        <v>43.20617210805162</v>
       </c>
     </row>
     <row r="30">
@@ -2664,10 +2664,10 @@
         <v>13</v>
       </c>
       <c r="S30" t="n">
-        <v>51.3913785253671</v>
+        <v>37.65486200795662</v>
       </c>
       <c r="T30" t="n">
-        <v>51.3913785253671</v>
+        <v>37.65486200795662</v>
       </c>
     </row>
     <row r="31">
@@ -2738,10 +2738,10 @@
         <v>13</v>
       </c>
       <c r="S31" t="n">
-        <v>50.24173524035834</v>
+        <v>36.59990325039727</v>
       </c>
       <c r="T31" t="n">
-        <v>50.24173524035834</v>
+        <v>36.59990325039727</v>
       </c>
     </row>
     <row r="32">
@@ -2812,10 +2812,10 @@
         <v>13</v>
       </c>
       <c r="S32" t="n">
-        <v>46.91903037262617</v>
+        <v>33.55085608532602</v>
       </c>
       <c r="T32" t="n">
-        <v>46.91903037262617</v>
+        <v>33.55085608532602</v>
       </c>
     </row>
     <row r="33">
@@ -2886,10 +2886,10 @@
         <v>13</v>
       </c>
       <c r="S33" t="n">
-        <v>39.84606147983398</v>
+        <v>27.06041633527854</v>
       </c>
       <c r="T33" t="n">
-        <v>39.84606147983398</v>
+        <v>27.06041633527854</v>
       </c>
     </row>
     <row r="34">
@@ -2960,10 +2960,10 @@
         <v>13</v>
       </c>
       <c r="S34" t="n">
-        <v>38.99434776501858</v>
+        <v>26.27884969274292</v>
       </c>
       <c r="T34" t="n">
-        <v>38.99434776501858</v>
+        <v>26.27884969274292</v>
       </c>
     </row>
     <row r="35">
@@ -3034,10 +3034,10 @@
         <v>13</v>
       </c>
       <c r="S35" t="n">
-        <v>32.86064717841157</v>
+        <v>20.65032018757669</v>
       </c>
       <c r="T35" t="n">
-        <v>32.86064717841157</v>
+        <v>20.65032018757669</v>
       </c>
     </row>
     <row r="36">
@@ -3108,10 +3108,10 @@
         <v>13</v>
       </c>
       <c r="S36" t="n">
-        <v>21.5711847073071</v>
+        <v>10.29065692738672</v>
       </c>
       <c r="T36" t="n">
-        <v>21.5711847073071</v>
+        <v>10.29065692738672</v>
       </c>
     </row>
     <row r="37">
@@ -3184,10 +3184,10 @@
         <v>0</v>
       </c>
       <c r="S37" t="n">
-        <v>91.55712447279947</v>
+        <v>74.51256038595842</v>
       </c>
       <c r="T37" t="n">
-        <v>91.55712447279947</v>
+        <v>74.51256038595842</v>
       </c>
     </row>
     <row r="38">
@@ -3258,10 +3258,10 @@
         <v>0</v>
       </c>
       <c r="S38" t="n">
-        <v>81.47851778194605</v>
+        <v>65.26402692244054</v>
       </c>
       <c r="T38" t="n">
-        <v>81.47851778194605</v>
+        <v>65.26402692244054</v>
       </c>
     </row>
     <row r="39">
@@ -3332,10 +3332,10 @@
         <v>0</v>
       </c>
       <c r="S39" t="n">
-        <v>87.51451396860166</v>
+        <v>70.80289895408876</v>
       </c>
       <c r="T39" t="n">
-        <v>87.51451396860166</v>
+        <v>70.80289895408876</v>
       </c>
     </row>
     <row r="40">
@@ -3406,10 +3406,10 @@
         <v>0</v>
       </c>
       <c r="S40" t="n">
-        <v>78.09478608084524</v>
+        <v>62.15897908903339</v>
       </c>
       <c r="T40" t="n">
-        <v>78.09478608084524</v>
+        <v>62.15897908903339</v>
       </c>
     </row>
     <row r="41">
@@ -3480,10 +3480,10 @@
         <v>0</v>
       </c>
       <c r="S41" t="n">
-        <v>74.34252922644359</v>
+        <v>58.71575780397802</v>
       </c>
       <c r="T41" t="n">
-        <v>74.34252922644359</v>
+        <v>58.71575780397802</v>
       </c>
     </row>
     <row r="42">
@@ -3554,10 +3554,10 @@
         <v>0</v>
       </c>
       <c r="S42" t="n">
-        <v>68.89840652149155</v>
+        <v>53.72001260221909</v>
       </c>
       <c r="T42" t="n">
-        <v>68.89840652149155</v>
+        <v>53.72001260221909</v>
       </c>
     </row>
     <row r="43">
@@ -3628,10 +3628,10 @@
         <v>0</v>
       </c>
       <c r="S43" t="n">
-        <v>75.28729356074702</v>
+        <v>59.58271142454872</v>
       </c>
       <c r="T43" t="n">
-        <v>75.28729356074702</v>
+        <v>59.58271142454872</v>
       </c>
     </row>
     <row r="44">
@@ -3702,10 +3702,10 @@
         <v>0</v>
       </c>
       <c r="S44" t="n">
-        <v>74.3012094153964</v>
+        <v>58.67784108920802</v>
       </c>
       <c r="T44" t="n">
-        <v>74.3012094153964</v>
+        <v>58.67784108920802</v>
       </c>
     </row>
     <row r="45">
@@ -3776,10 +3776,10 @@
         <v>0</v>
       </c>
       <c r="S45" t="n">
-        <v>79.08645331725144</v>
+        <v>63.06897269250443</v>
       </c>
       <c r="T45" t="n">
-        <v>79.08645331725144</v>
+        <v>63.06897269250443</v>
       </c>
     </row>
     <row r="46">
@@ -3850,10 +3850,10 @@
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>72.16822999909613</v>
+        <v>56.72053368415265</v>
       </c>
       <c r="T46" t="n">
-        <v>72.16822999909613</v>
+        <v>56.72053368415265</v>
       </c>
     </row>
     <row r="47">
@@ -3924,10 +3924,10 @@
         <v>0</v>
       </c>
       <c r="S47" t="n">
-        <v>74.97125440060455</v>
+        <v>59.29270122393118</v>
       </c>
       <c r="T47" t="n">
-        <v>74.97125440060455</v>
+        <v>59.29270122393118</v>
       </c>
     </row>
     <row r="48">
@@ -3998,10 +3998,10 @@
         <v>0</v>
       </c>
       <c r="S48" t="n">
-        <v>64.66929938134842</v>
+        <v>49.83921438217224</v>
       </c>
       <c r="T48" t="n">
-        <v>64.66929938134842</v>
+        <v>49.83921438217224</v>
       </c>
     </row>
     <row r="49">
@@ -4072,10 +4072,10 @@
         <v>0</v>
       </c>
       <c r="S49" t="n">
-        <v>58.48812636979474</v>
+        <v>44.16712227711689</v>
       </c>
       <c r="T49" t="n">
-        <v>58.48812636979474</v>
+        <v>44.16712227711689</v>
       </c>
     </row>
     <row r="50">
@@ -4146,10 +4146,10 @@
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>54.95921784379583</v>
+        <v>40.92885437030258</v>
       </c>
       <c r="T50" t="n">
-        <v>54.95921784379583</v>
+        <v>40.92885437030258</v>
       </c>
     </row>
     <row r="51">
@@ -4220,10 +4220,10 @@
         <v>0</v>
       </c>
       <c r="S51" t="n">
-        <v>56.07037639475384</v>
+        <v>41.94849799337753</v>
       </c>
       <c r="T51" t="n">
-        <v>56.07037639475384</v>
+        <v>41.94849799337753</v>
       </c>
     </row>
     <row r="52">
@@ -4366,10 +4366,10 @@
         <v>0</v>
       </c>
       <c r="S53" t="n">
-        <v>87.82178384030279</v>
+        <v>71.08486210414776</v>
       </c>
       <c r="T53" t="n">
-        <v>87.82178384030279</v>
+        <v>71.08486210414776</v>
       </c>
     </row>
     <row r="54">
@@ -4440,10 +4440,10 @@
         <v>0</v>
       </c>
       <c r="S54" t="n">
-        <v>86.57228009720134</v>
+        <v>69.93826738770228</v>
       </c>
       <c r="T54" t="n">
-        <v>86.57228009720134</v>
+        <v>69.93826738770228</v>
       </c>
     </row>
     <row r="55">
@@ -4514,10 +4514,10 @@
         <v>0</v>
       </c>
       <c r="S55" t="n">
-        <v>87.20597280663171</v>
+        <v>70.51976921712408</v>
       </c>
       <c r="T55" t="n">
-        <v>87.20597280663171</v>
+        <v>70.51976921712408</v>
       </c>
     </row>
     <row r="56">
@@ -4588,10 +4588,10 @@
         <v>0</v>
       </c>
       <c r="S56" t="n">
-        <v>83.82723527232726</v>
+        <v>67.41930423134215</v>
       </c>
       <c r="T56" t="n">
-        <v>83.82723527232726</v>
+        <v>67.41930423134215</v>
       </c>
     </row>
     <row r="57">
@@ -4662,10 +4662,10 @@
         <v>0</v>
       </c>
       <c r="S57" t="n">
-        <v>85.39372890754254</v>
+        <v>68.85678157816869</v>
       </c>
       <c r="T57" t="n">
-        <v>85.39372890754254</v>
+        <v>68.85678157816869</v>
       </c>
     </row>
     <row r="58">
@@ -4736,10 +4736,10 @@
         <v>0</v>
       </c>
       <c r="S58" t="n">
-        <v>78.49607118083193</v>
+        <v>62.52721438082288</v>
       </c>
       <c r="T58" t="n">
-        <v>78.49607118083193</v>
+        <v>62.52721438082288</v>
       </c>
     </row>
     <row r="59">
@@ -4810,10 +4810,10 @@
         <v>0</v>
       </c>
       <c r="S59" t="n">
-        <v>75.04724231747664</v>
+        <v>59.36243078215</v>
       </c>
       <c r="T59" t="n">
-        <v>75.04724231747664</v>
+        <v>59.36243078215</v>
       </c>
     </row>
     <row r="60">
@@ -4884,10 +4884,10 @@
         <v>0</v>
       </c>
       <c r="S60" t="n">
-        <v>75.76890803171716</v>
+        <v>60.0246601668609</v>
       </c>
       <c r="T60" t="n">
-        <v>75.76890803171716</v>
+        <v>60.0246601668609</v>
       </c>
     </row>
     <row r="61">
@@ -4958,10 +4958,10 @@
         <v>0</v>
       </c>
       <c r="S61" t="n">
-        <v>73.1640458649448</v>
+        <v>57.6343342362827</v>
       </c>
       <c r="T61" t="n">
-        <v>73.1640458649448</v>
+        <v>57.6343342362827</v>
       </c>
     </row>
     <row r="62">
@@ -5032,10 +5032,10 @@
         <v>0</v>
       </c>
       <c r="S62" t="n">
-        <v>74.27336694994455</v>
+        <v>58.65229172694625</v>
       </c>
       <c r="T62" t="n">
-        <v>74.27336694994455</v>
+        <v>58.65229172694625</v>
       </c>
     </row>
     <row r="63">
@@ -5106,10 +5106,10 @@
         <v>0</v>
       </c>
       <c r="S63" t="n">
-        <v>73.76341059684292</v>
+        <v>58.18433533760981</v>
       </c>
       <c r="T63" t="n">
-        <v>73.76341059684292</v>
+        <v>58.18433533760981</v>
       </c>
     </row>
     <row r="64">
@@ -5180,10 +5180,10 @@
         <v>0</v>
       </c>
       <c r="S64" t="n">
-        <v>72.07404182969069</v>
+        <v>56.63410284471883</v>
       </c>
       <c r="T64" t="n">
-        <v>72.07404182969069</v>
+        <v>56.63410284471883</v>
       </c>
     </row>
     <row r="65">
@@ -5254,10 +5254,10 @@
         <v>0</v>
       </c>
       <c r="S65" t="n">
-        <v>74.87273168184265</v>
+        <v>59.20229282827336</v>
       </c>
       <c r="T65" t="n">
-        <v>74.87273168184265</v>
+        <v>59.20229282827336</v>
       </c>
     </row>
     <row r="66">
@@ -5328,10 +5328,10 @@
         <v>0</v>
       </c>
       <c r="S66" t="n">
-        <v>61.88705494747212</v>
+        <v>47.28611537358176</v>
       </c>
       <c r="T66" t="n">
-        <v>61.88705494747212</v>
+        <v>47.28611537358176</v>
       </c>
     </row>
     <row r="67">
@@ -5402,10 +5402,10 @@
         <v>0</v>
       </c>
       <c r="S67" t="n">
-        <v>61.30700726531963</v>
+        <v>46.75384037135433</v>
       </c>
       <c r="T67" t="n">
-        <v>61.30700726531963</v>
+        <v>46.75384037135433</v>
       </c>
     </row>
     <row r="68">
@@ -5476,10 +5476,10 @@
         <v>0</v>
       </c>
       <c r="S68" t="n">
-        <v>53.66980214860921</v>
+        <v>39.74563484689951</v>
       </c>
       <c r="T68" t="n">
-        <v>53.66980214860921</v>
+        <v>39.74563484689951</v>
       </c>
     </row>
     <row r="69">
@@ -5552,10 +5552,10 @@
         <v>0</v>
       </c>
       <c r="S69" t="n">
-        <v>90.0367005711572</v>
+        <v>73.1173584731948</v>
       </c>
       <c r="T69" t="n">
-        <v>90.0367005711572</v>
+        <v>73.1173584731948</v>
       </c>
     </row>
     <row r="70">
@@ -5626,10 +5626,10 @@
         <v>0</v>
       </c>
       <c r="S70" t="n">
-        <v>89.52390857452765</v>
+        <v>72.64679998370075</v>
       </c>
       <c r="T70" t="n">
-        <v>89.52390857452765</v>
+        <v>72.64679998370075</v>
       </c>
     </row>
     <row r="71">
@@ -5700,10 +5700,10 @@
         <v>0</v>
       </c>
       <c r="S71" t="n">
-        <v>86.21337194025546</v>
+        <v>69.60891887737139</v>
       </c>
       <c r="T71" t="n">
-        <v>86.21337194025546</v>
+        <v>69.60891887737139</v>
       </c>
     </row>
     <row r="72">
@@ -5774,10 +5774,10 @@
         <v>0</v>
       </c>
       <c r="S72" t="n">
-        <v>86.58220042074608</v>
+        <v>69.94737067420672</v>
       </c>
       <c r="T72" t="n">
-        <v>86.58220042074608</v>
+        <v>69.94737067420672</v>
       </c>
     </row>
     <row r="73">
@@ -5848,10 +5848,10 @@
         <v>0</v>
       </c>
       <c r="S73" t="n">
-        <v>85.71966447306818</v>
+        <v>69.15587311702696</v>
       </c>
       <c r="T73" t="n">
-        <v>85.71966447306818</v>
+        <v>69.15587311702696</v>
       </c>
     </row>
     <row r="74">
@@ -5922,10 +5922,10 @@
         <v>0</v>
       </c>
       <c r="S74" t="n">
-        <v>87.88409448708416</v>
+        <v>71.14204085112813</v>
       </c>
       <c r="T74" t="n">
-        <v>87.88409448708416</v>
+        <v>71.14204085112813</v>
       </c>
     </row>
     <row r="75">
@@ -5996,10 +5996,10 @@
         <v>0</v>
       </c>
       <c r="S75" t="n">
-        <v>87.70777039166013</v>
+        <v>70.98023879386227</v>
       </c>
       <c r="T75" t="n">
-        <v>87.70777039166013</v>
+        <v>70.98023879386227</v>
       </c>
     </row>
     <row r="76">
@@ -6070,10 +6070,10 @@
         <v>0</v>
       </c>
       <c r="S76" t="n">
-        <v>83.07480304170771</v>
+        <v>66.72884225803885</v>
       </c>
       <c r="T76" t="n">
-        <v>83.07480304170771</v>
+        <v>66.72884225803885</v>
       </c>
     </row>
     <row r="77">
@@ -6144,10 +6144,10 @@
         <v>0</v>
       </c>
       <c r="S77" t="n">
-        <v>83.37164976412885</v>
+        <v>67.00124070854483</v>
       </c>
       <c r="T77" t="n">
-        <v>83.37164976412885</v>
+        <v>67.00124070854483</v>
       </c>
     </row>
     <row r="78">
@@ -6218,10 +6218,10 @@
         <v>0</v>
       </c>
       <c r="S78" t="n">
-        <v>84.00496438775549</v>
+        <v>67.58239559127894</v>
       </c>
       <c r="T78" t="n">
-        <v>84.00496438775549</v>
+        <v>67.58239559127894</v>
       </c>
     </row>
     <row r="79">
@@ -6292,10 +6292,10 @@
         <v>0</v>
       </c>
       <c r="S79" t="n">
-        <v>83.93298262968604</v>
+        <v>67.5163422449496</v>
       </c>
       <c r="T79" t="n">
-        <v>83.93298262968604</v>
+        <v>67.5163422449496</v>
       </c>
     </row>
     <row r="80">
@@ -6366,10 +6366,10 @@
         <v>0</v>
       </c>
       <c r="S80" t="n">
-        <v>80.0376722407148</v>
+        <v>63.94184930279683</v>
       </c>
       <c r="T80" t="n">
-        <v>80.0376722407148</v>
+        <v>63.94184930279683</v>
       </c>
     </row>
     <row r="81">
@@ -6440,10 +6440,10 @@
         <v>0</v>
       </c>
       <c r="S81" t="n">
-        <v>79.96569048264534</v>
+        <v>63.87579595646747</v>
       </c>
       <c r="T81" t="n">
-        <v>79.96569048264534</v>
+        <v>63.87579595646747</v>
       </c>
     </row>
     <row r="82">
@@ -6514,10 +6514,10 @@
         <v>0</v>
       </c>
       <c r="S82" t="n">
-        <v>79.78936638722132</v>
+        <v>63.71399389920161</v>
       </c>
       <c r="T82" t="n">
-        <v>79.78936638722132</v>
+        <v>63.71399389920161</v>
       </c>
     </row>
     <row r="83">
@@ -6588,10 +6588,10 @@
         <v>0</v>
       </c>
       <c r="S83" t="n">
-        <v>78.46693567154108</v>
+        <v>62.50047846970756</v>
       </c>
       <c r="T83" t="n">
-        <v>78.46693567154108</v>
+        <v>62.50047846970756</v>
       </c>
     </row>
     <row r="84">
@@ -6734,10 +6734,10 @@
         <v>0</v>
       </c>
       <c r="S85" t="n">
-        <v>63.04189449935333</v>
+        <v>48.34584243389658</v>
       </c>
       <c r="T85" t="n">
-        <v>63.04189449935333</v>
+        <v>48.34584243389658</v>
       </c>
     </row>
     <row r="86">
@@ -6808,10 +6808,10 @@
         <v>0</v>
       </c>
       <c r="S86" t="n">
-        <v>60.46200702618761</v>
+        <v>45.97843428319084</v>
       </c>
       <c r="T86" t="n">
-        <v>60.46200702618761</v>
+        <v>45.97843428319084</v>
       </c>
     </row>
     <row r="87">
@@ -6882,10 +6882,10 @@
         <v>0</v>
       </c>
       <c r="S87" t="n">
-        <v>59.60204453513237</v>
+        <v>45.18929823295559</v>
       </c>
       <c r="T87" t="n">
-        <v>59.60204453513237</v>
+        <v>45.18929823295559</v>
       </c>
     </row>
     <row r="88">
@@ -6956,10 +6956,10 @@
         <v>0</v>
       </c>
       <c r="S88" t="n">
-        <v>54.16325965928699</v>
+        <v>40.19845123713223</v>
       </c>
       <c r="T88" t="n">
-        <v>54.16325965928699</v>
+        <v>40.19845123713223</v>
       </c>
     </row>
     <row r="89">
@@ -7030,10 +7030,10 @@
         <v>0</v>
       </c>
       <c r="S89" t="n">
-        <v>50.72340969506602</v>
+        <v>37.04190703619125</v>
       </c>
       <c r="T89" t="n">
-        <v>50.72340969506602</v>
+        <v>37.04190703619125</v>
       </c>
     </row>
     <row r="90">
@@ -7104,10 +7104,10 @@
         <v>0</v>
       </c>
       <c r="S90" t="n">
-        <v>50.46542094774946</v>
+        <v>36.80516622112068</v>
       </c>
       <c r="T90" t="n">
-        <v>50.46542094774946</v>
+        <v>36.80516622112068</v>
       </c>
     </row>
     <row r="91">
@@ -7178,10 +7178,10 @@
         <v>0</v>
       </c>
       <c r="S91" t="n">
-        <v>50.03543970222183</v>
+        <v>36.41059819600305</v>
       </c>
       <c r="T91" t="n">
-        <v>50.03543970222183</v>
+        <v>36.41059819600305</v>
       </c>
     </row>
     <row r="92">
@@ -7252,10 +7252,10 @@
         <v>0</v>
       </c>
       <c r="S92" t="n">
-        <v>49.98384195275852</v>
+        <v>36.36325003298894</v>
       </c>
       <c r="T92" t="n">
-        <v>49.98384195275852</v>
+        <v>36.36325003298894</v>
       </c>
     </row>
     <row r="93">
@@ -7326,10 +7326,10 @@
         <v>0</v>
       </c>
       <c r="S93" t="n">
-        <v>47.83393572512042</v>
+        <v>34.39040990740082</v>
       </c>
       <c r="T93" t="n">
-        <v>47.83393572512042</v>
+        <v>34.39040990740082</v>
       </c>
     </row>
     <row r="94">
@@ -7400,10 +7400,10 @@
         <v>0</v>
       </c>
       <c r="S94" t="n">
-        <v>48.54292690016197</v>
+        <v>35.04100862693033</v>
       </c>
       <c r="T94" t="n">
-        <v>48.54292690016197</v>
+        <v>35.04100862693033</v>
       </c>
     </row>
     <row r="95">
@@ -7474,10 +7474,10 @@
         <v>0</v>
       </c>
       <c r="S95" t="n">
-        <v>47.25298316357912</v>
+        <v>33.85730455157746</v>
       </c>
       <c r="T95" t="n">
-        <v>47.25298316357912</v>
+        <v>33.85730455157746</v>
       </c>
     </row>
     <row r="96">
@@ -7548,10 +7548,10 @@
         <v>0</v>
       </c>
       <c r="S96" t="n">
-        <v>42.95317070830291</v>
+        <v>29.91162430040123</v>
       </c>
       <c r="T96" t="n">
-        <v>42.95317070830291</v>
+        <v>29.91162430040123</v>
       </c>
     </row>
     <row r="97">
@@ -7622,10 +7622,10 @@
         <v>0</v>
       </c>
       <c r="S97" t="n">
-        <v>38.65335825302671</v>
+        <v>25.965944049225</v>
       </c>
       <c r="T97" t="n">
-        <v>38.65335825302671</v>
+        <v>25.965944049225</v>
       </c>
     </row>
     <row r="98">
@@ -7698,10 +7698,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S98" t="n">
-        <v>58.08055862725779</v>
+        <v>43.79312178070658</v>
       </c>
       <c r="T98" t="n">
-        <v>58.08055862725779</v>
+        <v>43.79312178070658</v>
       </c>
     </row>
     <row r="99">
@@ -7772,10 +7772,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S99" t="n">
-        <v>61.95151403208638</v>
+        <v>47.34526561322983</v>
       </c>
       <c r="T99" t="n">
-        <v>61.95151403208638</v>
+        <v>47.34526561322983</v>
       </c>
     </row>
     <row r="100">
@@ -7846,10 +7846,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S100" t="n">
-        <v>61.00894667021709</v>
+        <v>46.48032802262228</v>
       </c>
       <c r="T100" t="n">
-        <v>61.00894667021709</v>
+        <v>46.48032802262228</v>
       </c>
     </row>
     <row r="101">
@@ -7920,10 +7920,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S101" t="n">
-        <v>59.72802427023176</v>
+        <v>45.30490228731851</v>
       </c>
       <c r="T101" t="n">
-        <v>59.72802427023176</v>
+        <v>45.30490228731851</v>
       </c>
     </row>
     <row r="102">
@@ -7994,10 +7994,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S102" t="n">
-        <v>50.35071467973962</v>
+        <v>36.69990715201472</v>
       </c>
       <c r="T102" t="n">
-        <v>50.35071467973962</v>
+        <v>36.69990715201472</v>
       </c>
     </row>
     <row r="103">
@@ -8068,10 +8068,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S103" t="n">
-        <v>58.27631221691505</v>
+        <v>43.97275312064089</v>
       </c>
       <c r="T103" t="n">
-        <v>58.27631221691505</v>
+        <v>43.97275312064089</v>
       </c>
     </row>
     <row r="104">
@@ -8142,10 +8142,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S104" t="n">
-        <v>52.99150576928252</v>
+        <v>39.12320290220629</v>
       </c>
       <c r="T104" t="n">
-        <v>52.99150576928252</v>
+        <v>39.12320290220629</v>
       </c>
     </row>
     <row r="105">
@@ -8216,10 +8216,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S105" t="n">
-        <v>48.51633804070067</v>
+        <v>35.0166096237717</v>
       </c>
       <c r="T105" t="n">
-        <v>48.51633804070067</v>
+        <v>35.0166096237717</v>
       </c>
     </row>
     <row r="106">
@@ -8290,10 +8290,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S106" t="n">
-        <v>54.73726331310906</v>
+        <v>40.72517999671095</v>
       </c>
       <c r="T106" t="n">
-        <v>54.73726331310906</v>
+        <v>40.72517999671095</v>
       </c>
     </row>
     <row r="107">
@@ -8364,10 +8364,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S107" t="n">
-        <v>53.75038640363356</v>
+        <v>39.8195821892342</v>
       </c>
       <c r="T107" t="n">
-        <v>53.75038640363356</v>
+        <v>39.8195821892342</v>
       </c>
     </row>
     <row r="108">
@@ -8438,10 +8438,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S108" t="n">
-        <v>50.08485739410238</v>
+        <v>36.45594585079961</v>
       </c>
       <c r="T108" t="n">
-        <v>50.08485739410238</v>
+        <v>36.45594585079961</v>
       </c>
     </row>
     <row r="109">
@@ -8512,10 +8512,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S109" t="n">
-        <v>47.09603846080327</v>
+        <v>33.71328580175746</v>
       </c>
       <c r="T109" t="n">
-        <v>47.09603846080327</v>
+        <v>33.71328580175746</v>
       </c>
     </row>
     <row r="110">
@@ -8586,10 +8586,10 @@
         <v>10.55515787799252</v>
       </c>
       <c r="S110" t="n">
-        <v>33.61010438471792</v>
+        <v>21.33805215932724</v>
       </c>
       <c r="T110" t="n">
-        <v>33.61010438471792</v>
+        <v>21.33805215932724</v>
       </c>
     </row>
   </sheetData>

</xml_diff>